<commit_message>
option to generate nadir
</commit_message>
<xml_diff>
--- a/dataset/create_dataset/dataset_overview.xlsx
+++ b/dataset/create_dataset/dataset_overview.xlsx
@@ -439,7 +439,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ocean</t>
+          <t>full</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1"/>
@@ -603,7 +603,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Pelagos2016/PelagosIm4_FW_WV3_PS_20160619_B2.PNG</t>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -624,241 +624,29 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>PelagosIm4_FW_WV3_PS_20160619_B2_1</t>
+          <t>Ignacio_GW_WV3_PS_20170220_B0_1</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>ocean</t>
+          <t>whale</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>64</v>
+        <v>42</v>
       </c>
       <c r="J3" t="n">
-        <v>3</v>
+        <v>28</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>[0.04187192118226601]</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Pelagos2016/PelagosIm4_FW_WV3_PS_20160619_B2.PNG</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>TC_1x1sat_30deg_5min_1sd</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>4648171f-6db2-4cd9-b02d-5ddbed392445</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>13</v>
-      </c>
-      <c r="F4" t="n">
-        <v>43</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>PelagosIm4_FW_WV3_PS_20160619_B2_2</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>ocean</t>
-        </is>
-      </c>
-      <c r="I4" t="n">
-        <v>64</v>
-      </c>
-      <c r="J4" t="n">
-        <v>3</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>[0.04187192118226601]</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Pelagos2016/PelagosIm4_FW_WV3_PS_20160619_B2.PNG</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>TC_1x1sat_40deg_9min_17sd</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>35ba1fc8-d20f-4be9-9b7f-d3f7b9743be8</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>14</v>
-      </c>
-      <c r="F5" t="n">
-        <v>44</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>PelagosIm4_FW_WV3_PS_20160619_B2_3</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>ocean</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>64</v>
-      </c>
-      <c r="J5" t="n">
-        <v>13</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="n">
-        <v>1</v>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>[0.09113300492610837]</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Pelagos2016/PelagosIm4_FW_WV3_PS_20160619_B2.PNG</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>TC_1x1sat_60deg_5min_1sd</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>efe0a2b6-adad-43e9-8218-7c1a557175f2</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>15</v>
-      </c>
-      <c r="F6" t="n">
-        <v>45</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>PelagosIm4_FW_WV3_PS_20160619_B2_4</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>ocean</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>64</v>
-      </c>
-      <c r="J6" t="n">
-        <v>3</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="n">
-        <v>1</v>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>[0.04187192118226601]</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Pelagos2016/PelagosIm4_FW_WV3_PS_20160619_B2.PNG</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>TC_1x1sat_30deg_5min_17sd</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>c5f4d7d1-55cf-425f-97ee-06c5a8f13d50</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>16</v>
-      </c>
-      <c r="F7" t="n">
-        <v>46</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>PelagosIm4_FW_WV3_PS_20160619_B2_5</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>ocean</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>64</v>
-      </c>
-      <c r="J7" t="n">
-        <v>7</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="n">
-        <v>1</v>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>[0.06157635467980296]</t>
+          <t>[1.0]</t>
         </is>
       </c>
     </row>
@@ -873,7 +661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1"/>
@@ -940,7 +728,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Pelagos2016/PelagosIm4_FW_WV3_PS_20160619_B2.PNG</t>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -970,162 +758,6 @@
       <c r="K3" t="inlineStr">
         <is>
           <t>2025-09-20T12:59:15Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Pelagos2016/PelagosIm4_FW_WV3_PS_20160619_B2.PNG</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" t="n">
-        <v>18</v>
-      </c>
-      <c r="E4" t="n">
-        <v>56.63394232326019</v>
-      </c>
-      <c r="F4" t="n">
-        <v>-168.0852787553452</v>
-      </c>
-      <c r="G4" t="n">
-        <v>623209.7933165799</v>
-      </c>
-      <c r="H4" t="n">
-        <v>53.35397450406396</v>
-      </c>
-      <c r="I4" t="n">
-        <v>-168.9457725713284</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>2025-09-20T22:31:05Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Pelagos2016/PelagosIm4_FW_WV3_PS_20160619_B2.PNG</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D5" t="n">
-        <v>19</v>
-      </c>
-      <c r="E5" t="n">
-        <v>-11.93706662739639</v>
-      </c>
-      <c r="F5" t="n">
-        <v>7.484415709841971</v>
-      </c>
-      <c r="G5" t="n">
-        <v>614159.8806786895</v>
-      </c>
-      <c r="H5" t="n">
-        <v>-16.18683795939982</v>
-      </c>
-      <c r="I5" t="n">
-        <v>9.931777464040437</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>2025-09-20T09:53:27Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Pelagos2016/PelagosIm4_FW_WV3_PS_20160619_B2.PNG</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D6" t="n">
-        <v>20</v>
-      </c>
-      <c r="E6" t="n">
-        <v>-27.49394307872987</v>
-      </c>
-      <c r="F6" t="n">
-        <v>-44.54360775652795</v>
-      </c>
-      <c r="G6" t="n">
-        <v>618521.2889087405</v>
-      </c>
-      <c r="H6" t="n">
-        <v>-25.59928124466757</v>
-      </c>
-      <c r="I6" t="n">
-        <v>-42.45696638790653</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>2025-09-20T13:11:44Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Pelagos2016/PelagosIm4_FW_WV3_PS_20160619_B2.PNG</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>5</v>
-      </c>
-      <c r="D7" t="n">
-        <v>21</v>
-      </c>
-      <c r="E7" t="n">
-        <v>18.89080344868408</v>
-      </c>
-      <c r="F7" t="n">
-        <v>155.642470545997</v>
-      </c>
-      <c r="G7" t="n">
-        <v>612601.5976574868</v>
-      </c>
-      <c r="H7" t="n">
-        <v>15.65395030985926</v>
-      </c>
-      <c r="I7" t="n">
-        <v>155.2570075274126</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>2025-09-21T00:18:26Z</t>
         </is>
       </c>
     </row>
@@ -1140,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1"/>
@@ -1207,204 +839,40 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Pelagos2016/PelagosIm4_FW_WV3_PS_20160619_B2.PNG</t>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PelagosIm4_FW_WV3_PS_20160619_B2_1</t>
+          <t>Ignacio_GW_WV3_PS_20170220_B0_1</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>267</v>
+        <v>104</v>
       </c>
       <c r="E3" t="n">
-        <v>298</v>
+        <v>108</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>[0.0, 41.0, 1.0, 23.0]</t>
+          <t>[1.0, 31.0, 31.717, 19.557999999999993]</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>[[0.0, 64.0, 1.0, 64.0, 1.0, 61.0, 0.0, 61.0, 0.0, 50.0, 0.0, 50.0]]</t>
+          <t>[[0.8560000000000016, 36.971000000000004, 1.134999999999998, 40.602999999999994, 6.164999999999999, 41.301, 13.430999999999997, 40.32299999999999, 13.151000000000003, 43.537000000000006, 15.665999999999997, 47.867000000000004, 18.180999999999997, 50.242000000000004, 23.909999999999997, 50.661, 27.543000000000006, 46.888999999999996, 29.638999999999996, 42.559, 32.57299999999999, 39.066, 31.873999999999995, 35.294, 26.983999999999995, 32.919, 22.373000000000005, 32.919, 18.880000000000003, 32.081, 13.430999999999997, 31.662, 6.584000000000003, 31.103, 3.1480000000000032, 33.564, 0.8560000000000016, 36.971000000000004]]</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>560</v>
+        <v>620.321</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
       </c>
       <c r="K3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Pelagos2016/PelagosIm4_FW_WV3_PS_20160619_B2.PNG</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>PelagosIm4_FW_WV3_PS_20160619_B2_2</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>267</v>
-      </c>
-      <c r="E4" t="n">
-        <v>298</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>[0.0, 41.0, 1.0, 23.0]</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>[[0.0, 64.0, 1.0, 64.0, 1.0, 61.0, 0.0, 61.0, 0.0, 50.0, 0.0, 50.0]]</t>
-        </is>
-      </c>
-      <c r="I4" t="n">
-        <v>560</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Pelagos2016/PelagosIm4_FW_WV3_PS_20160619_B2.PNG</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>PelagosIm4_FW_WV3_PS_20160619_B2_3</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>267</v>
-      </c>
-      <c r="E5" t="n">
-        <v>298</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>[0.0, 31.0, 1.0, 33.0]</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>[[0.0, 64.0, 1.0, 64.0, 1.0, 51.0, 0.0, 51.0, 0.0, 40.0, 0.0, 40.0]]</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>560</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Pelagos2016/PelagosIm4_FW_WV3_PS_20160619_B2.PNG</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>PelagosIm4_FW_WV3_PS_20160619_B2_4</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>267</v>
-      </c>
-      <c r="E6" t="n">
-        <v>298</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>[0.0, 41.0, 1.0, 23.0]</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>[[0.0, 64.0, 1.0, 64.0, 1.0, 61.0, 0.0, 61.0, 0.0, 50.0, 0.0, 50.0]]</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>560</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Pelagos2016/PelagosIm4_FW_WV3_PS_20160619_B2.PNG</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>PelagosIm4_FW_WV3_PS_20160619_B2_5</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>267</v>
-      </c>
-      <c r="E7" t="n">
-        <v>298</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>[0.0, 37.0, 1.0, 27.0]</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>[[0.0, 64.0, 1.0, 64.0, 1.0, 57.0, 0.0, 57.0, 0.0, 46.0, 0.0, 46.0]]</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>560</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Generate nadir image with sunglint
</commit_message>
<xml_diff>
--- a/dataset/create_dataset/dataset_overview.xlsx
+++ b/dataset/create_dataset/dataset_overview.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1"/>
@@ -645,6 +645,218 @@
         <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
+        <is>
+          <t>[1.0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TC_1x1sat_30deg_5min_1sd</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>4648171f-6db2-4cd9-b02d-5ddbed392445</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>13</v>
+      </c>
+      <c r="F4" t="n">
+        <v>43</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Ignacio_GW_WV3_PS_20170220_B0_2</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>whale</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>32</v>
+      </c>
+      <c r="J4" t="n">
+        <v>42</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>[1.0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TC_1x1sat_40deg_9min_17sd</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>35ba1fc8-d20f-4be9-9b7f-d3f7b9743be8</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>14</v>
+      </c>
+      <c r="F5" t="n">
+        <v>44</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Ignacio_GW_WV3_PS_20170220_B0_3</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>whale</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>43</v>
+      </c>
+      <c r="J5" t="n">
+        <v>26</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>[0.995049504950495]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TC_1x1sat_60deg_5min_1sd</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>efe0a2b6-adad-43e9-8218-7c1a557175f2</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>15</v>
+      </c>
+      <c r="F6" t="n">
+        <v>45</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Ignacio_GW_WV3_PS_20170220_B0_4</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>whale</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>34</v>
+      </c>
+      <c r="J6" t="n">
+        <v>49</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>[1.0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>TC_1x1sat_30deg_5min_17sd</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>c5f4d7d1-55cf-425f-97ee-06c5a8f13d50</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>16</v>
+      </c>
+      <c r="F7" t="n">
+        <v>46</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Ignacio_GW_WV3_PS_20170220_B0_5</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>whale</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>32</v>
+      </c>
+      <c r="J7" t="n">
+        <v>58</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="inlineStr">
         <is>
           <t>[1.0]</t>
         </is>
@@ -661,7 +873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1"/>
@@ -758,6 +970,162 @@
       <c r="K3" t="inlineStr">
         <is>
           <t>2025-09-20T12:59:15Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>18</v>
+      </c>
+      <c r="E4" t="n">
+        <v>56.63394232326019</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-168.0852787553452</v>
+      </c>
+      <c r="G4" t="n">
+        <v>623209.7933165799</v>
+      </c>
+      <c r="H4" t="n">
+        <v>53.35397450406396</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-168.9457725713284</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2025-09-20T22:31:05Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" t="n">
+        <v>19</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-11.93706662739639</v>
+      </c>
+      <c r="F5" t="n">
+        <v>7.484415709841971</v>
+      </c>
+      <c r="G5" t="n">
+        <v>614159.8806786895</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-16.18683795939982</v>
+      </c>
+      <c r="I5" t="n">
+        <v>9.931777464040437</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2025-09-20T09:53:27Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-27.49394307872987</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-44.54360775652795</v>
+      </c>
+      <c r="G6" t="n">
+        <v>618521.2889087405</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-25.59928124466757</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-42.45696638790653</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2025-09-20T13:11:44Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D7" t="n">
+        <v>21</v>
+      </c>
+      <c r="E7" t="n">
+        <v>18.89080344868408</v>
+      </c>
+      <c r="F7" t="n">
+        <v>155.642470545997</v>
+      </c>
+      <c r="G7" t="n">
+        <v>612601.5976574868</v>
+      </c>
+      <c r="H7" t="n">
+        <v>15.65395030985926</v>
+      </c>
+      <c r="I7" t="n">
+        <v>155.2570075274126</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2025-09-21T00:18:26Z</t>
         </is>
       </c>
     </row>
@@ -772,7 +1140,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1"/>
@@ -874,6 +1242,170 @@
       </c>
       <c r="K3" t="inlineStr"/>
     </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Ignacio_GW_WV3_PS_20170220_B0_2</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>104</v>
+      </c>
+      <c r="E4" t="n">
+        <v>108</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>[11.0, 17.0, 31.717, 19.557999999999993]</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>[[10.856000000000002, 22.971000000000004, 11.134999999999998, 26.602999999999994, 16.165, 27.301000000000002, 23.430999999999997, 26.322999999999993, 23.151000000000003, 29.537000000000006, 25.665999999999997, 33.867000000000004, 28.180999999999997, 36.242000000000004, 33.91, 36.661, 37.543000000000006, 32.888999999999996, 39.638999999999996, 28.558999999999997, 42.57299999999999, 25.066000000000003, 41.873999999999995, 21.293999999999997, 36.983999999999995, 18.918999999999997, 32.373000000000005, 18.918999999999997, 28.880000000000003, 18.081000000000003, 23.430999999999997, 17.662, 16.584000000000003, 17.103, 13.148000000000003, 19.564, 10.856000000000002, 22.971000000000004]]</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>620.321</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Ignacio_GW_WV3_PS_20170220_B0_3</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>104</v>
+      </c>
+      <c r="E5" t="n">
+        <v>108</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>[0.0, 33.0, 31.717, 19.557999999999993]</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>[[0.0, 40.84558064516129, 0.134999999999998, 42.602999999999994, 5.164999999999999, 43.301, 12.430999999999997, 42.32299999999999, 12.151000000000003, 45.537000000000006, 14.665999999999997, 49.867000000000004, 17.180999999999997, 52.242000000000004, 22.909999999999997, 52.661, 26.543000000000006, 48.888999999999996, 28.638999999999996, 44.559, 31.572999999999993, 41.066, 30.873999999999995, 37.294, 25.983999999999995, 34.919, 21.373000000000005, 34.919, 17.880000000000003, 34.081, 12.430999999999997, 33.662, 5.584000000000003, 33.103, 2.1480000000000032, 35.564, 0.0, 38.75694764397906]]</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>620.321</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Ignacio_GW_WV3_PS_20170220_B0_4</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>104</v>
+      </c>
+      <c r="E6" t="n">
+        <v>108</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>[9.0, 10.0, 31.717, 19.557999999999993]</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>[[8.856000000000002, 15.971000000000004, 9.134999999999998, 19.602999999999994, 14.165, 20.301000000000002, 21.430999999999997, 19.322999999999993, 21.151000000000003, 22.537000000000006, 23.665999999999997, 26.867000000000004, 26.180999999999997, 29.242000000000004, 31.909999999999997, 29.661, 35.543000000000006, 25.888999999999996, 37.638999999999996, 21.558999999999997, 40.57299999999999, 18.066000000000003, 39.873999999999995, 14.293999999999997, 34.983999999999995, 11.918999999999997, 30.373000000000005, 11.918999999999997, 26.880000000000003, 11.081000000000003, 21.430999999999997, 10.661999999999999, 14.584000000000003, 10.103000000000002, 11.148000000000003, 12.564, 8.856000000000002, 15.971000000000004]]</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>620.321</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Ignacio_GW_WV3_PS_20170220_B0_5</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>104</v>
+      </c>
+      <c r="E7" t="n">
+        <v>108</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>[11.0, 1.0, 31.717, 19.557999999999993]</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>[[10.856000000000002, 6.971000000000004, 11.134999999999998, 10.602999999999994, 16.165, 11.301000000000002, 23.430999999999997, 10.322999999999993, 23.151000000000003, 13.537000000000006, 25.665999999999997, 17.867000000000004, 28.180999999999997, 20.242000000000004, 33.91, 20.661, 37.543000000000006, 16.888999999999996, 39.638999999999996, 12.558999999999997, 42.57299999999999, 9.066000000000003, 41.873999999999995, 5.293999999999997, 36.983999999999995, 2.918999999999997, 32.373000000000005, 2.918999999999997, 28.880000000000003, 2.081000000000003, 23.430999999999997, 1.661999999999999, 16.584000000000003, 1.1030000000000015, 13.148000000000003, 3.564, 10.856000000000002, 6.971000000000004]]</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>620.321</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
create dataset scripts completed
</commit_message>
<xml_diff>
--- a/dataset/create_dataset/dataset_overview.xlsx
+++ b/dataset/create_dataset/dataset_overview.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1"/>
@@ -645,6 +645,218 @@
         <v>0</v>
       </c>
       <c r="M3" t="inlineStr">
+        <is>
+          <t>[1.0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TC_1x1sat_30deg_5min_1sd</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>4648171f-6db2-4cd9-b02d-5ddbed392445</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>13</v>
+      </c>
+      <c r="F4" t="n">
+        <v>43</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Ignacio_GW_WV3_PS_20170220_B0_2</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>whale</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>32</v>
+      </c>
+      <c r="J4" t="n">
+        <v>42</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>[1.0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TC_1x1sat_40deg_9min_17sd</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>35ba1fc8-d20f-4be9-9b7f-d3f7b9743be8</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>14</v>
+      </c>
+      <c r="F5" t="n">
+        <v>44</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Ignacio_GW_WV3_PS_20170220_B0_3</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>whale</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>43</v>
+      </c>
+      <c r="J5" t="n">
+        <v>26</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>[0.995049504950495]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TC_1x1sat_60deg_5min_1sd</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>efe0a2b6-adad-43e9-8218-7c1a557175f2</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>15</v>
+      </c>
+      <c r="F6" t="n">
+        <v>45</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Ignacio_GW_WV3_PS_20170220_B0_4</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>whale</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>34</v>
+      </c>
+      <c r="J6" t="n">
+        <v>49</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>[1.0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>TC_1x1sat_30deg_5min_17sd</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>c5f4d7d1-55cf-425f-97ee-06c5a8f13d50</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>16</v>
+      </c>
+      <c r="F7" t="n">
+        <v>46</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Ignacio_GW_WV3_PS_20170220_B0_5</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>whale</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>32</v>
+      </c>
+      <c r="J7" t="n">
+        <v>58</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="inlineStr">
         <is>
           <t>[1.0]</t>
         </is>
@@ -661,7 +873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1"/>
@@ -758,6 +970,162 @@
       <c r="K3" t="inlineStr">
         <is>
           <t>2025-09-20T12:59:15Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>18</v>
+      </c>
+      <c r="E4" t="n">
+        <v>56.63394232326019</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-168.0852787553452</v>
+      </c>
+      <c r="G4" t="n">
+        <v>623209.7933165799</v>
+      </c>
+      <c r="H4" t="n">
+        <v>53.35397450406396</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-168.9457725713284</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2025-09-20T22:31:05Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" t="n">
+        <v>19</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-11.93706662739639</v>
+      </c>
+      <c r="F5" t="n">
+        <v>7.484415709841971</v>
+      </c>
+      <c r="G5" t="n">
+        <v>614159.8806786895</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-16.18683795939982</v>
+      </c>
+      <c r="I5" t="n">
+        <v>9.931777464040437</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2025-09-20T09:53:27Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-27.49394307872987</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-44.54360775652795</v>
+      </c>
+      <c r="G6" t="n">
+        <v>618521.2889087405</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-25.59928124466757</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-42.45696638790653</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2025-09-20T13:11:44Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D7" t="n">
+        <v>21</v>
+      </c>
+      <c r="E7" t="n">
+        <v>18.89080344868408</v>
+      </c>
+      <c r="F7" t="n">
+        <v>155.642470545997</v>
+      </c>
+      <c r="G7" t="n">
+        <v>612601.5976574868</v>
+      </c>
+      <c r="H7" t="n">
+        <v>15.65395030985926</v>
+      </c>
+      <c r="I7" t="n">
+        <v>155.2570075274126</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2025-09-21T00:18:26Z</t>
         </is>
       </c>
     </row>
@@ -772,7 +1140,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1"/>
@@ -874,6 +1242,170 @@
       </c>
       <c r="K3" t="inlineStr"/>
     </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Ignacio_GW_WV3_PS_20170220_B0_2</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>104</v>
+      </c>
+      <c r="E4" t="n">
+        <v>108</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>[11.0, 17.0, 31.717, 19.557999999999993]</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>[[10.856000000000002, 22.971000000000004, 11.134999999999998, 26.602999999999994, 16.165, 27.301000000000002, 23.430999999999997, 26.322999999999993, 23.151000000000003, 29.537000000000006, 25.665999999999997, 33.867000000000004, 28.180999999999997, 36.242000000000004, 33.91, 36.661, 37.543000000000006, 32.888999999999996, 39.638999999999996, 28.558999999999997, 42.57299999999999, 25.066000000000003, 41.873999999999995, 21.293999999999997, 36.983999999999995, 18.918999999999997, 32.373000000000005, 18.918999999999997, 28.880000000000003, 18.081000000000003, 23.430999999999997, 17.662, 16.584000000000003, 17.103, 13.148000000000003, 19.564, 10.856000000000002, 22.971000000000004]]</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>620.321</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Ignacio_GW_WV3_PS_20170220_B0_3</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>104</v>
+      </c>
+      <c r="E5" t="n">
+        <v>108</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>[0.0, 33.0, 31.717, 19.557999999999993]</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>[[0.0, 40.84558064516129, 0.134999999999998, 42.602999999999994, 5.164999999999999, 43.301, 12.430999999999997, 42.32299999999999, 12.151000000000003, 45.537000000000006, 14.665999999999997, 49.867000000000004, 17.180999999999997, 52.242000000000004, 22.909999999999997, 52.661, 26.543000000000006, 48.888999999999996, 28.638999999999996, 44.559, 31.572999999999993, 41.066, 30.873999999999995, 37.294, 25.983999999999995, 34.919, 21.373000000000005, 34.919, 17.880000000000003, 34.081, 12.430999999999997, 33.662, 5.584000000000003, 33.103, 2.1480000000000032, 35.564, 0.0, 38.75694764397906]]</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>620.321</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Ignacio_GW_WV3_PS_20170220_B0_4</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>104</v>
+      </c>
+      <c r="E6" t="n">
+        <v>108</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>[9.0, 10.0, 31.717, 19.557999999999993]</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>[[8.856000000000002, 15.971000000000004, 9.134999999999998, 19.602999999999994, 14.165, 20.301000000000002, 21.430999999999997, 19.322999999999993, 21.151000000000003, 22.537000000000006, 23.665999999999997, 26.867000000000004, 26.180999999999997, 29.242000000000004, 31.909999999999997, 29.661, 35.543000000000006, 25.888999999999996, 37.638999999999996, 21.558999999999997, 40.57299999999999, 18.066000000000003, 39.873999999999995, 14.293999999999997, 34.983999999999995, 11.918999999999997, 30.373000000000005, 11.918999999999997, 26.880000000000003, 11.081000000000003, 21.430999999999997, 10.661999999999999, 14.584000000000003, 10.103000000000002, 11.148000000000003, 12.564, 8.856000000000002, 15.971000000000004]]</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>620.321</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ignacio2017/Ignacio_GW_WV3_PS_20170220_B0.PNG</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Ignacio_GW_WV3_PS_20170220_B0_5</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>104</v>
+      </c>
+      <c r="E7" t="n">
+        <v>108</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>[11.0, 1.0, 31.717, 19.557999999999993]</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>[[10.856000000000002, 6.971000000000004, 11.134999999999998, 10.602999999999994, 16.165, 11.301000000000002, 23.430999999999997, 10.322999999999993, 23.151000000000003, 13.537000000000006, 25.665999999999997, 17.867000000000004, 28.180999999999997, 20.242000000000004, 33.91, 20.661, 37.543000000000006, 16.888999999999996, 39.638999999999996, 12.558999999999997, 42.57299999999999, 9.066000000000003, 41.873999999999995, 5.293999999999997, 36.983999999999995, 2.918999999999997, 32.373000000000005, 2.918999999999997, 28.880000000000003, 2.081000000000003, 23.430999999999997, 1.661999999999999, 16.584000000000003, 1.1030000000000015, 13.148000000000003, 3.564, 10.856000000000002, 6.971000000000004]]</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>620.321</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
add off nadir tags to name
</commit_message>
<xml_diff>
--- a/dataset/create_dataset/dataset_overview.xlsx
+++ b/dataset/create_dataset/dataset_overview.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1"/>
@@ -709,6 +709,118 @@
         <v>-90</v>
       </c>
       <c r="N4" t="inlineStr">
+        <is>
+          <t>[1.0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Maui2015/Maui_HB_WV3_PS_20150109_B1.PNG</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TC_1x1sat_15deg_5min_17sd</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ad1caca4-503a-4ef4-b712-a9c3d5007185</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>12</v>
+      </c>
+      <c r="F5" t="n">
+        <v>44</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Maui_HB_WV3_PS_20150109_B1_3</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>whale</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>25</v>
+      </c>
+      <c r="J5" t="n">
+        <v>44</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" t="n">
+        <v>90</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>[1.0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Maui2015/Maui_HB_WV3_PS_20150109_B1.PNG</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TC_1x1sat_20deg_5min_17sd</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>91a591c5-bb58-43a4-8f26-fcabc030066a</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>12</v>
+      </c>
+      <c r="F6" t="n">
+        <v>45</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Maui_HB_WV3_PS_20150109_B1_4</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>whale</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>34</v>
+      </c>
+      <c r="J6" t="n">
+        <v>49</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="inlineStr">
         <is>
           <t>[1.0]</t>
         </is>
@@ -725,7 +837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1"/>
@@ -873,6 +985,90 @@
       </c>
       <c r="L4" t="n">
         <v>11.11759847967619</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Maui2015/Maui_HB_WV3_PS_20150109_B1.PNG</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" t="n">
+        <v>19</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-39.49638431529891</v>
+      </c>
+      <c r="F5" t="n">
+        <v>49.24933025484319</v>
+      </c>
+      <c r="G5" t="n">
+        <v>623569.4176167186</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-41.02001209546279</v>
+      </c>
+      <c r="I5" t="n">
+        <v>49.0800580641276</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2025-09-20T06:46:52Z</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>16.70682747059459</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Maui2015/Maui_HB_WV3_PS_20150109_B1.PNG</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4.694489889798024</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-110.3524889039977</v>
+      </c>
+      <c r="G6" t="n">
+        <v>611961.4160458741</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2.62030645552691</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-110.3807330453514</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2025-09-20T17:54:08Z</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>22.49086164226176</v>
       </c>
     </row>
   </sheetData>
@@ -886,7 +1082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1"/>
@@ -1029,6 +1225,88 @@
       </c>
       <c r="K4" t="inlineStr"/>
     </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Maui2015/Maui_HB_WV3_PS_20150109_B1.PNG</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Maui_HB_WV3_PS_20150109_B1_3</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>185</v>
+      </c>
+      <c r="E5" t="n">
+        <v>720</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>[14.0, 10.0, 43.0, 38.0]</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>[[14.0, 34.0, 21.0, 40.0, 33.0, 47.0, 46.0, 48.0, 53.0, 39.0, 57.0, 26.0, 50.0, 16.0, 39.0, 14.0, 33.0, 10.0, 25.0, 13.0, 18.0, 18.0, 14.0, 27.0]]</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>1634</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Maui2015/Maui_HB_WV3_PS_20150109_B1.PNG</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Maui_HB_WV3_PS_20150109_B1_4</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>185</v>
+      </c>
+      <c r="E6" t="n">
+        <v>720</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>[5.0, 5.0, 43.0, 38.0]</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>[[5.0, 29.0, 12.0, 35.0, 24.0, 42.0, 37.0, 43.0, 44.0, 34.0, 48.0, 21.0, 41.0, 11.0, 30.0, 9.0, 24.0, 5.0, 16.0, 8.0, 9.0, 13.0, 5.0, 22.0]]</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>1634</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>